<commit_message>
feat(stacktab): style block header rows in Excel composites (v1.8.5)
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_stacktab.xlsx
+++ b/tabtools/demo/demo_stacktab.xlsx
@@ -16,7 +16,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="67" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="67" uniqueCount="35">
+  <si>
+    <t>Source block: Primary HRT exposure model</t>
+  </si>
   <si>
     <t/>
   </si>
@@ -55,6 +58,9 @@
   </si>
   <si>
     <t>(1.21, 1.77)</t>
+  </si>
+  <si>
+    <t>Source block: Estrogen dose-response model</t>
   </si>
   <si>
     <t>Low dose</t>
@@ -108,1432 +114,1516 @@
     <t>aHR = adjusted hazard ratio; CI = confidence interval. Models adjusted for age and comorbidities.</t>
   </si>
   <si>
-    <t>Primary and Dose-Response Estimates Side by Side</t>
+    <t>Primary model</t>
+  </si>
+  <si>
+    <t>Dose-response model</t>
+  </si>
+  <si>
+    <t>Table 2 supplement. Primary and dose-response estimates side by side</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="487">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
+  <fonts count="483">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1891,205 +1981,119 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="12"/>
@@ -2145,7 +2149,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="390">
+  <borders count="386">
     <border>
       <left/>
       <right/>
@@ -4025,6 +4029,90 @@
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
     <border/>
     <border/>
     <border>
@@ -4447,48 +4535,6 @@
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -4551,64 +4597,6 @@
     <border/>
     <border/>
     <border/>
-    <border/>
-    <border/>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -4754,7 +4742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="390">
+  <cellXfs count="386">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -5830,57 +5818,60 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="277" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="278" xfId="0"/>
-    <xf numFmtId="0" fontId="344" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="346" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="348" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="349" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="350" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="351" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="352" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="353" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="354" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="356" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="358" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="360" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="291" xfId="0"/>
+    <xf numFmtId="0" fontId="344" fillId="0" borderId="277" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="346" fillId="0" borderId="278" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="347" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="348" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="349" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="350" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="352" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="354" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="355" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="356" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="357" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="358" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="289" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="290" xfId="0"/>
+    <xf numFmtId="0" fontId="360" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="0" fontId="362" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5898,175 +5889,172 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="367" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="368" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="370" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="372" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="300" xfId="0"/>
+    <xf numFmtId="0" fontId="369" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="370" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="372" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="0" fontId="374" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="376" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="378" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="380" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="382" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="384" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="386" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="388" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="390" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="392" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="394" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="396" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="397" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="398" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="399" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="400" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="401" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="402" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="403" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="303" xfId="0"/>
+    <xf numFmtId="0" fontId="378" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="380" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="381" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="382" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="383" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="384" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="386" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="388" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="312" xfId="0"/>
+    <xf numFmtId="0" fontId="390" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="392" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="394" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="396" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="398" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="400" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="402" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="404" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="405" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="406" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="407" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="408" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="409" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="410" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="411" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="412" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="413" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="414" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="415" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="416" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="417" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="418" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="419" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="420" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="422" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="424" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="426" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="406" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="408" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="410" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="412" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="413" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="414" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="415" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="416" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="417" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="418" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="419" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="420" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="421" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="422" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="423" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="424" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="425" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="426" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="427" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6074,39 +6062,39 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="430" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="432" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="433" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="434" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="435" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="436" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="437" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="438" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="439" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="429" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="430" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="431" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="432" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="433" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="434" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="435" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="436" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="438" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6114,44 +6102,50 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="441" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="442" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="443" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="444" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="355" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="356" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="357" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="358" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="359" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="360" xfId="0"/>
-    <xf numFmtId="0" fontId="446" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="448" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="450" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="452" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="442" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="444" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="445" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="446" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="447" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="448" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="449" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="450" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="451" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="452" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="361" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="362" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="363" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="364" xfId="0"/>
     <xf numFmtId="0" fontId="454" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6164,91 +6158,75 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="459" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="460" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="461" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="462" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="463" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="464" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="465" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="466" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="467" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="468" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="469" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="470" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="471" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="472" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="474" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="476" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="478" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="480" fillId="0" borderId="385" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="482" fillId="0" borderId="386" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="484" fillId="0" borderId="387" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="486" fillId="0" borderId="388" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="389" xfId="0"/>
+    <xf numFmtId="0" fontId="460" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="462" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="463" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="464" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="465" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="466" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="467" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="468" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="469" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="470" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="471" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="472" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="474" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="476" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="478" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="480" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="482" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="385" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6272,69 +6250,69 @@
         <v>0</v>
       </c>
       <c r="B1" s="96" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="97" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D1" s="98" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="69" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="109" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="110" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="111" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="73" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="74" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="112" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="113" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="77" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="78" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="114" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="115" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="81" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" s="118" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="119" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="120" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -6357,58 +6335,58 @@
   <sheetData>
     <row r="1" s="189" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="203" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B1" s="200" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="201" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D1" s="202" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="177" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="213" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="214" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="215" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="181" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="182" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" s="216" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="217" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="185" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="221" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="222" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -6423,86 +6401,86 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="18.7109375" style="277" customWidth="true"/>
-    <col min="3" max="3" width="19.7109375" style="278" customWidth="true"/>
+    <col min="2" max="2" width="18.7109375" style="289" customWidth="true"/>
+    <col min="3" max="3" width="19.7109375" style="290" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="291" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="288" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="289"/>
-      <c r="C1" s="290"/>
+    <row r="1" s="303" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="300" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="301"/>
+      <c r="C1" s="302"/>
     </row>
     <row r="2">
-      <c r="B2" s="273" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="274" t="s">
+      <c r="B2" s="281" t="s">
         <v>21</v>
+      </c>
+      <c r="C2" s="282" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="257" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="258" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="259" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="260" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="261" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="262" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="263" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="264" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="265" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="266" t="s">
-        <v>25</v>
+      <c r="B7" s="287" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="288" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="267" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" s="268" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="275" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C9" s="276" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
-    <row r="10" s="300" customFormat="true" ht="45" customHeight="true">
-      <c r="B10" s="298" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="299"/>
+    <row r="10" s="312" customFormat="true" ht="45" customHeight="true">
+      <c r="B10" s="310" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="311"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6514,71 +6492,69 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="15.7109375" style="355" customWidth="true"/>
-    <col min="3" max="3" width="10.7109375" style="356" customWidth="true"/>
-    <col min="4" max="4" width="14.7109375" style="357" customWidth="true"/>
-    <col min="5" max="5" width="11.7109375" style="358" customWidth="true"/>
-    <col min="6" max="6" width="10.7109375" style="359" customWidth="true"/>
-    <col min="7" max="7" width="14.7109375" style="360" customWidth="true"/>
+    <col min="2" max="2" width="15.7109375" style="361" customWidth="true"/>
+    <col min="3" max="3" width="19.7109375" style="362" customWidth="true"/>
+    <col min="4" max="4" width="21.7109375" style="363" customWidth="true"/>
+    <col min="5" max="5" width="19.7109375" style="364" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="389" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="382" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="383"/>
-      <c r="C1" s="384"/>
-      <c r="D1" s="385"/>
-      <c r="E1" s="386"/>
-      <c r="F1" s="387"/>
-      <c r="G1" s="388"/>
+    <row r="1" s="385" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="380" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="381"/>
+      <c r="C1" s="382"/>
+      <c r="D1" s="383"/>
+      <c r="E1" s="384"/>
     </row>
     <row r="2">
-      <c r="B2" s="343" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="344" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="345" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="346" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="347" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="348" t="s">
-        <v>17</v>
+      <c r="B2" s="353" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="354" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="355" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="356" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="349" t="s">
+      <c r="B3" s="341" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="350" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="351" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="352" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="353" t="s">
+      <c r="C3" s="342" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="343" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="344" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="357" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="358" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="359" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="354" t="s">
-        <v>18</v>
+      <c r="E4" s="360" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(qa): add xlsx checker tool and refresh QA tests and demos
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_stacktab.xlsx
+++ b/tabtools/demo/demo_stacktab.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="67" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="65" uniqueCount="35">
   <si>
     <t>Source block: Primary HRT exposure model</t>
   </si>
@@ -127,1274 +127,1242 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="483">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+  <fonts count="475">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2149,7 +2117,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="386">
+  <borders count="380">
     <border>
       <left/>
       <right/>
@@ -3963,48 +3931,6 @@
       <left style="none"/>
       <right style="none"/>
       <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
@@ -4742,7 +4668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="386">
+  <cellXfs count="380">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -5658,119 +5584,119 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="300" fillId="0" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="302" fillId="0" borderId="238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="303" fillId="0" borderId="239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="304" fillId="0" borderId="240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="305" fillId="0" borderId="241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="306" fillId="0" borderId="242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="307" fillId="0" borderId="243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="308" fillId="0" borderId="244" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="309" fillId="0" borderId="245" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="310" fillId="0" borderId="246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="311" fillId="0" borderId="247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="312" fillId="0" borderId="248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="313" fillId="0" borderId="249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="314" fillId="0" borderId="250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="315" fillId="0" borderId="251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="316" fillId="0" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="317" fillId="0" borderId="253" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="318" fillId="0" borderId="254" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="319" fillId="0" borderId="255" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="320" fillId="0" borderId="256" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="321" fillId="0" borderId="257" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="322" fillId="0" borderId="258" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="323" fillId="0" borderId="259" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="324" fillId="0" borderId="260" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="325" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="326" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="327" fillId="0" borderId="263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="328" fillId="0" borderId="264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="329" fillId="0" borderId="265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="299" fillId="0" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="300" fillId="0" borderId="238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="301" fillId="0" borderId="239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="302" fillId="0" borderId="240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="303" fillId="0" borderId="241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="304" fillId="0" borderId="242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="305" fillId="0" borderId="243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="306" fillId="0" borderId="244" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="307" fillId="0" borderId="245" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="308" fillId="0" borderId="246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="309" fillId="0" borderId="247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="310" fillId="0" borderId="248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="311" fillId="0" borderId="249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="312" fillId="0" borderId="250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="313" fillId="0" borderId="251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="314" fillId="0" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="315" fillId="0" borderId="253" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="316" fillId="0" borderId="254" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="317" fillId="0" borderId="255" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="318" fillId="0" borderId="256" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="319" fillId="0" borderId="257" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="320" fillId="0" borderId="258" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="321" fillId="0" borderId="259" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="322" fillId="0" borderId="260" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="323" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="324" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="325" fillId="0" borderId="263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="326" fillId="0" borderId="264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="328" fillId="0" borderId="265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5842,235 +5768,235 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="352" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="354" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="355" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="356" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="357" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="358" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="289" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="290" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="283" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="284" xfId="0"/>
+    <xf numFmtId="0" fontId="352" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="354" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="356" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="357" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="358" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="359" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="0" fontId="360" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="362" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="364" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="365" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="361" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="362" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="364" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="366" fillId="0" borderId="295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="367" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="368" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="369" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="370" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="372" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="368" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="297" xfId="0"/>
+    <xf numFmtId="0" fontId="370" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="372" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="373" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="374" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="376" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="303" xfId="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="375" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="376" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="0" fontId="378" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="380" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="381" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="306" xfId="0"/>
     <xf numFmtId="0" fontId="382" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="383" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="384" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="386" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="388" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="312" xfId="0"/>
-    <xf numFmtId="0" fontId="390" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="392" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="394" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="396" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="398" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="400" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="402" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="404" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="406" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="384" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="386" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="388" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="390" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="392" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="394" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="396" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="398" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="400" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="402" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="404" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="405" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="406" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="407" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="408" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="410" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="412" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="413" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="414" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="415" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="416" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="417" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="418" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="419" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="420" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="421" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="422" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="423" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="424" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="425" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="426" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="427" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="428" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="429" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="430" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="431" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="409" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="410" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="411" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="412" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="413" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="414" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="415" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="416" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="417" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="418" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="419" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="420" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="421" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="422" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="423" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="424" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="425" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="426" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="427" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="428" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="430" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6078,23 +6004,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="433" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="434" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="435" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="436" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="438" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="434" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="436" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="437" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="438" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="439" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6102,131 +6028,107 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="442" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="444" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="445" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="446" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="447" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="448" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="449" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="450" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="451" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="452" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="361" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="362" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="363" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="364" xfId="0"/>
-    <xf numFmtId="0" fontId="454" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="456" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="441" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="442" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="443" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="444" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="355" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="356" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="357" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="358" xfId="0"/>
+    <xf numFmtId="0" fontId="446" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="448" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="450" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="452" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="454" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="455" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="456" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="457" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="458" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="460" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="462" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="463" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="464" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="465" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="466" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="467" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="459" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="460" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="461" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="462" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="463" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="464" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="466" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="468" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="469" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="470" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="471" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="472" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="474" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="476" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="478" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="480" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="482" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="385" xfId="0"/>
+    <xf numFmtId="0" fontId="470" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="472" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="474" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="379" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6398,94 +6300,86 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="18.7109375" style="289" customWidth="true"/>
-    <col min="3" max="3" width="19.7109375" style="290" customWidth="true"/>
+    <col min="2" max="2" width="18.7109375" style="283" customWidth="true"/>
+    <col min="3" max="3" width="19.7109375" style="284" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="303" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="300" t="s">
+    <row r="1" s="297" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="294" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="301"/>
-      <c r="C1" s="302"/>
+      <c r="B1" s="295"/>
+      <c r="C1" s="296"/>
     </row>
     <row r="2">
-      <c r="B2" s="281" t="s">
+      <c r="B2" s="275" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="282" t="s">
+      <c r="C2" s="276" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="257" t="s">
+      <c r="B3" s="253" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="258" t="s">
+      <c r="C3" s="254" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="259" t="s">
+      <c r="B4" s="255" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="260" t="s">
+      <c r="C4" s="256" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="261" t="s">
+      <c r="B5" s="257" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="262" t="s">
+      <c r="C5" s="258" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="263" t="s">
-        <v>1</v>
+      <c r="B6" s="281" t="s">
+        <v>22</v>
       </c>
-      <c r="C6" s="264" t="s">
-        <v>1</v>
+      <c r="C6" s="282" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="287" t="s">
-        <v>22</v>
+      <c r="B7" s="261" t="s">
+        <v>15</v>
       </c>
-      <c r="C7" s="288" t="s">
-        <v>27</v>
+      <c r="C7" s="262" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="267" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="268" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="275" t="s">
+      <c r="B8" s="269" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="276" t="s">
+      <c r="C8" s="270" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" s="312" customFormat="true" ht="45" customHeight="true">
-      <c r="B10" s="310" t="s">
+    <row r="9" s="306" customFormat="true" ht="45" customHeight="true">
+      <c r="B9" s="304" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="311"/>
+      <c r="C9" s="305"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B9:C9"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -6495,60 +6389,60 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="15.7109375" style="361" customWidth="true"/>
-    <col min="3" max="3" width="19.7109375" style="362" customWidth="true"/>
-    <col min="4" max="4" width="21.7109375" style="363" customWidth="true"/>
-    <col min="5" max="5" width="19.7109375" style="364" customWidth="true"/>
+    <col min="2" max="2" width="15.7109375" style="355" customWidth="true"/>
+    <col min="3" max="3" width="19.7109375" style="356" customWidth="true"/>
+    <col min="4" max="4" width="21.7109375" style="357" customWidth="true"/>
+    <col min="5" max="5" width="19.7109375" style="358" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="385" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="380" t="s">
+    <row r="1" s="379" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="374" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="381"/>
-      <c r="C1" s="382"/>
-      <c r="D1" s="383"/>
-      <c r="E1" s="384"/>
+      <c r="B1" s="375"/>
+      <c r="C1" s="376"/>
+      <c r="D1" s="377"/>
+      <c r="E1" s="378"/>
     </row>
     <row r="2">
-      <c r="B2" s="353" t="s">
+      <c r="B2" s="347" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="354" t="s">
+      <c r="C2" s="348" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="355" t="s">
+      <c r="D2" s="349" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="356" t="s">
+      <c r="E2" s="350" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="341" t="s">
+      <c r="B3" s="335" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="342" t="s">
+      <c r="C3" s="336" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="343" t="s">
+      <c r="D3" s="337" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="344" t="s">
+      <c r="E3" s="338" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="357" t="s">
+      <c r="B4" s="351" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="358" t="s">
+      <c r="C4" s="352" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="359" t="s">
+      <c r="D4" s="353" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="360" t="s">
+      <c r="E4" s="354" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>